<commit_message>
Revisiones y correcciones sexta entrega
</commit_message>
<xml_diff>
--- a/Listado de prácticas.xlsx
+++ b/Listado de prácticas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DISCO D\Francisco\Trabajos\FCE\Optativa\UNL-Programacion-en-R\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositorios\UNL-Programacion-en-R\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11844E5E-5E90-444B-A905-24A2D26A821F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2A78415-C0D0-4E65-8B9A-46398BDD199D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -80,34 +80,6 @@
         </r>
       </text>
     </comment>
-    <comment ref="H12" authorId="0" shapeId="0" xr:uid="{BAC2716D-1FF6-4460-89A0-0563EA2A9792}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Error: `path` does not exist: ‘Growth.xlsx’</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I12" authorId="0" shapeId="0" xr:uid="{452042C0-E791-466A-BF82-179BD80140AB}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Error: `path` does not exist: ‘Growth.xlsx’</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="F13" authorId="0" shapeId="0" xr:uid="{3254A794-DC4A-404E-831A-F9197FDD3E71}">
       <text>
         <r>
@@ -119,21 +91,6 @@
             <family val="2"/>
           </rPr>
           <t>No corrió bien el codigo</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H18" authorId="0" shapeId="0" xr:uid="{CEEDE685-C6D5-416F-82DE-962D277B8B88}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>No pude corregir por falta de base de datos. Recomiendo enviar la msima para que pueda corregir el código
-Error: objeto 'ventas_autos_caba' no encontrado</t>
         </r>
       </text>
     </comment>
@@ -156,6 +113,25 @@
       </text>
     </comment>
     <comment ref="I20" authorId="0" shapeId="0" xr:uid="{54D00BC5-4CFA-4C7A-82D0-B8A12BA3A15C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>No pude corregir por falta de base de datos. Recomiendo enviar la msima para que pueda corregir el código
+&gt; datos_wdi &lt;- read.csv("datos_wdi.csv") # Cargo mi base de datos
+Error en file(file, "rt"): no se puede abrir la conexión
+Además: Aviso:
+In file(file, "rt") :
+  no fue posible abrir el archivo 'datos_wdi.csv': No such file or directory</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J20" authorId="0" shapeId="0" xr:uid="{AD638E5F-F377-4990-A421-8B88BEA4915C}">
       <text>
         <r>
           <rPr>
@@ -218,6 +194,36 @@
         </r>
       </text>
     </comment>
+    <comment ref="I24" authorId="0" shapeId="0" xr:uid="{33B50290-8D37-4F06-96A2-21AC55948CD4}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>No pude corregir por falta de base de datos. Recomiendo enviar la msima para que pueda corregir el código
+Error: `path` does not exist: ‘encuesta_poblacional.xlsx’</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J24" authorId="0" shapeId="0" xr:uid="{C660C20F-CB5E-4C04-8846-FC5D4594AB5A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>No pude corregir por falta de base de datos. Recomiendo enviar la msima para que pueda corregir el código
+Error: `path` does not exist: ‘encuesta_poblacional.xlsx’</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="I25" authorId="0" shapeId="0" xr:uid="{96B6402A-D9AF-46D1-A7DC-5FEE2CA79E1B}">
       <text>
         <r>
@@ -242,29 +248,12 @@
         </r>
       </text>
     </comment>
-    <comment ref="I26" authorId="0" shapeId="0" xr:uid="{B386A6A9-0E43-4783-9890-65DB365F7508}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>No pude corregir por falta de base de datos. Recomiendo enviar la msima para que pueda corregir el código
-Error: `path` does not exist: ‘Lista_de_clientes_con_nombre_y_direccion’
-&gt; clientes &lt;- read_excel("C:/ruta/Lista-de-clientes-con-nombre-y-direccion.xls")
-Error: `path` does not exist: ‘C:/ruta/Lista-de-clientes-con-nombre-y-direccion.xls’</t>
-        </r>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="29">
   <si>
     <t>Alumnos:</t>
   </si>
@@ -654,7 +643,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -952,12 +951,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:N28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="H2" s="22" t="s">
         <v>7</v>
       </c>
@@ -965,13 +964,13 @@
       <c r="J2" s="23"/>
       <c r="K2" s="24"/>
     </row>
-    <row r="3" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="20">
-        <v>45943.378472222219</v>
+        <v>45949.817361111112</v>
       </c>
       <c r="E3" s="21"/>
       <c r="H3" s="11" t="s">
@@ -983,8 +982,8 @@
       <c r="J3" s="12"/>
       <c r="K3" s="13"/>
     </row>
-    <row r="5" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="6" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="17" t="s">
         <v>0</v>
       </c>
@@ -1003,7 +1002,7 @@
       <c r="M6" s="25"/>
       <c r="N6" s="26"/>
     </row>
-    <row r="7" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="18"/>
       <c r="C7" s="4"/>
       <c r="D7" s="9">
@@ -1028,7 +1027,7 @@
       <c r="M7" s="9"/>
       <c r="N7" s="16"/>
     </row>
-    <row r="8" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B8" s="19"/>
       <c r="C8" s="6"/>
       <c r="D8" s="7">
@@ -1075,7 +1074,7 @@
         <v>45964</v>
       </c>
     </row>
-    <row r="9" spans="2:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:14" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="B9" s="5" t="s">
         <v>3</v>
       </c>
@@ -1102,7 +1101,7 @@
       <c r="M9" s="9"/>
       <c r="N9" s="10"/>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B10" s="5" t="s">
         <v>22</v>
       </c>
@@ -1123,13 +1122,15 @@
       <c r="I10" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="9"/>
+      <c r="J10" s="9" t="s">
+        <v>12</v>
+      </c>
       <c r="K10" s="9"/>
       <c r="L10" s="9"/>
       <c r="M10" s="9"/>
       <c r="N10" s="10"/>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B11" s="5" t="s">
         <v>17</v>
       </c>
@@ -1156,7 +1157,7 @@
       <c r="M11" s="9"/>
       <c r="N11" s="10"/>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B12" s="5" t="s">
         <v>5</v>
       </c>
@@ -1172,18 +1173,20 @@
       </c>
       <c r="G12" s="15"/>
       <c r="H12" s="9" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="J12" s="9"/>
+        <v>11</v>
+      </c>
+      <c r="J12" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="K12" s="9"/>
       <c r="L12" s="9"/>
       <c r="M12" s="9"/>
       <c r="N12" s="10"/>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B13" s="5" t="s">
         <v>27</v>
       </c>
@@ -1208,7 +1211,7 @@
       <c r="M13" s="9"/>
       <c r="N13" s="10"/>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B14" s="5" t="s">
         <v>13</v>
       </c>
@@ -1229,13 +1232,15 @@
       <c r="I14" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="J14" s="9"/>
+      <c r="J14" s="14" t="s">
+        <v>26</v>
+      </c>
       <c r="K14" s="9"/>
       <c r="L14" s="9"/>
       <c r="M14" s="9"/>
       <c r="N14" s="10"/>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B15" s="5" t="s">
         <v>20</v>
       </c>
@@ -1258,7 +1263,7 @@
       <c r="M15" s="9"/>
       <c r="N15" s="10"/>
     </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B16" s="5" t="s">
         <v>21</v>
       </c>
@@ -1285,7 +1290,7 @@
       <c r="M16" s="9"/>
       <c r="N16" s="10"/>
     </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B17" s="5" t="s">
         <v>9</v>
       </c>
@@ -1306,13 +1311,15 @@
       <c r="I17" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="J17" s="9"/>
+      <c r="J17" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="K17" s="9"/>
       <c r="L17" s="9"/>
       <c r="M17" s="9"/>
       <c r="N17" s="10"/>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B18" s="5" t="s">
         <v>6</v>
       </c>
@@ -1328,16 +1335,18 @@
       </c>
       <c r="G18" s="15"/>
       <c r="H18" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="I18" s="9"/>
+        <v>12</v>
+      </c>
+      <c r="I18" s="9" t="s">
+        <v>12</v>
+      </c>
       <c r="J18" s="9"/>
       <c r="K18" s="9"/>
       <c r="L18" s="9"/>
       <c r="M18" s="9"/>
       <c r="N18" s="10"/>
     </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B19" s="5" t="s">
         <v>1</v>
       </c>
@@ -1358,13 +1367,15 @@
       <c r="I19" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J19" s="9"/>
+      <c r="J19" s="9" t="s">
+        <v>11</v>
+      </c>
       <c r="K19" s="9"/>
       <c r="L19" s="9"/>
       <c r="M19" s="9"/>
       <c r="N19" s="10"/>
     </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B20" s="5" t="s">
         <v>16</v>
       </c>
@@ -1385,13 +1396,15 @@
       <c r="I20" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="J20" s="9"/>
+      <c r="J20" s="9" t="s">
+        <v>4</v>
+      </c>
       <c r="K20" s="9"/>
       <c r="L20" s="9"/>
       <c r="M20" s="9"/>
       <c r="N20" s="10"/>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B21" s="5" t="s">
         <v>18</v>
       </c>
@@ -1412,13 +1425,15 @@
       <c r="I21" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="J21" s="9"/>
+      <c r="J21" s="9" t="s">
+        <v>12</v>
+      </c>
       <c r="K21" s="9"/>
       <c r="L21" s="9"/>
       <c r="M21" s="9"/>
       <c r="N21" s="10"/>
     </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B22" s="5" t="s">
         <v>25</v>
       </c>
@@ -1445,7 +1460,7 @@
       <c r="M22" s="9"/>
       <c r="N22" s="10"/>
     </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B23" s="5" t="s">
         <v>24</v>
       </c>
@@ -1466,13 +1481,15 @@
       <c r="I23" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J23" s="9"/>
+      <c r="J23" s="14" t="s">
+        <v>12</v>
+      </c>
       <c r="K23" s="9"/>
       <c r="L23" s="9"/>
       <c r="M23" s="9"/>
       <c r="N23" s="10"/>
     </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B24" s="5" t="s">
         <v>23</v>
       </c>
@@ -1490,14 +1507,18 @@
       <c r="H24" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
+      <c r="I24" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="J24" s="9" t="s">
+        <v>4</v>
+      </c>
       <c r="K24" s="9"/>
       <c r="L24" s="9"/>
       <c r="M24" s="9"/>
       <c r="N24" s="10"/>
     </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B25" s="5" t="s">
         <v>14</v>
       </c>
@@ -1524,7 +1545,7 @@
       <c r="M25" s="9"/>
       <c r="N25" s="10"/>
     </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B26" s="5" t="s">
         <v>10</v>
       </c>
@@ -1543,15 +1564,17 @@
         <v>12</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="J26" s="9"/>
+        <v>12</v>
+      </c>
+      <c r="J26" s="9" t="s">
+        <v>11</v>
+      </c>
       <c r="K26" s="9"/>
       <c r="L26" s="9"/>
       <c r="M26" s="9"/>
       <c r="N26" s="10"/>
     </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B27" s="5" t="s">
         <v>19</v>
       </c>
@@ -1578,7 +1601,7 @@
       <c r="M27" s="9"/>
       <c r="N27" s="10"/>
     </row>
-    <row r="28" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B28" s="5" t="s">
         <v>15</v>
       </c>
@@ -1614,12 +1637,12 @@
     <mergeCell ref="D6:N6"/>
   </mergeCells>
   <conditionalFormatting sqref="D9:N28">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"R"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3">
-    <cfRule type="cellIs" dxfId="0" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="23" operator="equal">
       <formula>"R"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Correcciones 13 del 10
</commit_message>
<xml_diff>
--- a/Listado de prácticas.xlsx
+++ b/Listado de prácticas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Trabajos\Optativa-FCE\UNL-Programacion-en-R\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositorios\UNL-Programacion-en-R\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD0D12FA-F5EF-48CA-AA83-9EDB4B0BECDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE6AB190-328D-47D1-9D14-3DB5FF7CA5F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3840" yWindow="3840" windowWidth="12075" windowHeight="9585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -28,9 +28,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -83,7 +80,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J11" authorId="0" shapeId="0" xr:uid="{732E58AD-62D5-45A9-AB95-29428AF3A087}">
+    <comment ref="K11" authorId="0" shapeId="0" xr:uid="{732E58AD-62D5-45A9-AB95-29428AF3A087}">
       <text>
         <r>
           <rPr>
@@ -141,7 +138,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H24" authorId="0" shapeId="0" xr:uid="{FABC9E6E-5273-4913-8085-012620829B29}">
+    <comment ref="H24" authorId="0" shapeId="0" xr:uid="{429BE6B8-851B-49BB-B40B-30EF9FF9EDED}">
       <text>
         <r>
           <rPr>
@@ -151,12 +148,21 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>No pude corregir por falta de base de datos. Recomiendo enviar la msima para que pueda corregir el código
-Error: `path` does not exist: ‘encuesta_poblacional.xlsx’</t>
+          <t>&gt; g3 &lt;- ggplot(tabla, aes(x = "", y = Freq, fill = factor(Month))) +
++   geom_bar(stat = "identity", width = 1) +
++   coord_polar(theta = "y") +
++   labs(
++     title = "Proporción de observaciones por Mes",
++     fill = "Mes"
++   ) +
++   theme_void()
+Error: objeto 'tabla' no encontrado
+&gt; ggplotly(g3)
+Error: objeto 'Freq' no encontrado</t>
         </r>
       </text>
     </comment>
-    <comment ref="I24" authorId="0" shapeId="0" xr:uid="{33B50290-8D37-4F06-96A2-21AC55948CD4}">
+    <comment ref="I24" authorId="0" shapeId="0" xr:uid="{BAC1A85C-9A41-494E-AED5-8B137ABE4520}">
       <text>
         <r>
           <rPr>
@@ -166,23 +172,17 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>No pude corregir por falta de base de datos. Recomiendo enviar la msima para que pueda corregir el código
-Error: `path` does not exist: ‘encuesta_poblacional.xlsx’</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J24" authorId="0" shapeId="0" xr:uid="{C660C20F-CB5E-4C04-8846-FC5D4594AB5A}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>No pude corregir por falta de base de datos. Recomiendo enviar la msima para que pueda corregir el código
-Error: `path` does not exist: ‘encuesta_poblacional.xlsx’</t>
+          <t>&gt; g3 &lt;- ggplot(tabla, aes(x = "", y = Freq, fill = factor(Month))) +
++   geom_bar(stat = "identity", width = 1) +
++   coord_polar(theta = "y") +
++   labs(
++     title = "Proporción de observaciones por Mes",
++     fill = "Mes"
++   ) +
++   theme_void()
+Error: objeto 'tabla' no encontrado
+&gt; ggplotly(g3)
+Error: objeto 'Freq' no encontrado</t>
         </r>
       </text>
     </comment>
@@ -210,27 +210,12 @@
         </r>
       </text>
     </comment>
-    <comment ref="J25" authorId="0" shapeId="0" xr:uid="{D573ADB5-B073-425E-BEB7-C9A1B7C9BB50}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Falta enviar base de datos
-</t>
-        </r>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="29">
   <si>
     <t>Alumnos:</t>
   </si>
@@ -937,7 +922,7 @@
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="20">
-        <v>45950.029861111114</v>
+        <v>45952.691666666666</v>
       </c>
       <c r="E3" s="21"/>
       <c r="H3" s="11" t="s">
@@ -989,8 +974,12 @@
         <v>5</v>
       </c>
       <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
+      <c r="K7" s="9">
+        <v>6</v>
+      </c>
+      <c r="L7" s="9">
+        <v>7</v>
+      </c>
       <c r="M7" s="9"/>
       <c r="N7" s="16"/>
     </row>
@@ -1062,8 +1051,10 @@
       <c r="I9" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="9" t="s">
+        <v>11</v>
+      </c>
       <c r="L9" s="9"/>
       <c r="M9" s="9"/>
       <c r="N9" s="10"/>
@@ -1089,10 +1080,10 @@
       <c r="I10" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="K10" s="9"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="9" t="s">
+        <v>12</v>
+      </c>
       <c r="L10" s="9"/>
       <c r="M10" s="9"/>
       <c r="N10" s="10"/>
@@ -1118,10 +1109,10 @@
       <c r="I11" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J11" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="K11" s="9"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="9" t="s">
+        <v>12</v>
+      </c>
       <c r="L11" s="9"/>
       <c r="M11" s="9"/>
       <c r="N11" s="10"/>
@@ -1147,10 +1138,10 @@
       <c r="I12" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="J12" s="9" t="s">
+      <c r="J12" s="15"/>
+      <c r="K12" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="K12" s="9"/>
       <c r="L12" s="9"/>
       <c r="M12" s="9"/>
       <c r="N12" s="10"/>
@@ -1174,7 +1165,7 @@
         <v>12</v>
       </c>
       <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
+      <c r="J13" s="15"/>
       <c r="K13" s="9"/>
       <c r="L13" s="9"/>
       <c r="M13" s="9"/>
@@ -1201,10 +1192,10 @@
       <c r="I14" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="J14" s="14" t="s">
+      <c r="J14" s="15"/>
+      <c r="K14" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="K14" s="9"/>
       <c r="L14" s="9"/>
       <c r="M14" s="9"/>
       <c r="N14" s="10"/>
@@ -1226,7 +1217,7 @@
       <c r="G15" s="15"/>
       <c r="H15" s="9"/>
       <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
+      <c r="J15" s="15"/>
       <c r="K15" s="9"/>
       <c r="L15" s="9"/>
       <c r="M15" s="9"/>
@@ -1253,7 +1244,7 @@
       <c r="I16" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="J16" s="9"/>
+      <c r="J16" s="15"/>
       <c r="K16" s="9"/>
       <c r="L16" s="9"/>
       <c r="M16" s="9"/>
@@ -1280,10 +1271,10 @@
       <c r="I17" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="J17" s="9" t="s">
+      <c r="J17" s="15"/>
+      <c r="K17" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="K17" s="9"/>
       <c r="L17" s="9"/>
       <c r="M17" s="9"/>
       <c r="N17" s="10"/>
@@ -1309,7 +1300,7 @@
       <c r="I18" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J18" s="9"/>
+      <c r="J18" s="15"/>
       <c r="K18" s="9"/>
       <c r="L18" s="9"/>
       <c r="M18" s="9"/>
@@ -1336,10 +1327,10 @@
       <c r="I19" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J19" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="K19" s="9"/>
+      <c r="J19" s="15"/>
+      <c r="K19" s="9" t="s">
+        <v>11</v>
+      </c>
       <c r="L19" s="9"/>
       <c r="M19" s="9"/>
       <c r="N19" s="10"/>
@@ -1365,10 +1356,10 @@
       <c r="I20" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J20" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="K20" s="9"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="9" t="s">
+        <v>11</v>
+      </c>
       <c r="L20" s="9"/>
       <c r="M20" s="9"/>
       <c r="N20" s="10"/>
@@ -1394,10 +1385,10 @@
       <c r="I21" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="J21" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="K21" s="9"/>
+      <c r="J21" s="15"/>
+      <c r="K21" s="9" t="s">
+        <v>12</v>
+      </c>
       <c r="L21" s="9"/>
       <c r="M21" s="9"/>
       <c r="N21" s="10"/>
@@ -1423,7 +1414,7 @@
       <c r="I22" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="J22" s="9"/>
+      <c r="J22" s="15"/>
       <c r="K22" s="9"/>
       <c r="L22" s="9"/>
       <c r="M22" s="9"/>
@@ -1450,10 +1441,10 @@
       <c r="I23" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J23" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="K23" s="9"/>
+      <c r="J23" s="15"/>
+      <c r="K23" s="14" t="s">
+        <v>12</v>
+      </c>
       <c r="L23" s="9"/>
       <c r="M23" s="9"/>
       <c r="N23" s="10"/>
@@ -1474,15 +1465,15 @@
       </c>
       <c r="G24" s="15"/>
       <c r="H24" s="9" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="J24" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="K24" s="9"/>
+        <v>12</v>
+      </c>
+      <c r="J24" s="15"/>
+      <c r="K24" s="9" t="s">
+        <v>11</v>
+      </c>
       <c r="L24" s="9"/>
       <c r="M24" s="9"/>
       <c r="N24" s="10"/>
@@ -1508,10 +1499,10 @@
       <c r="I25" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J25" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="K25" s="9"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="9" t="s">
+        <v>12</v>
+      </c>
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
       <c r="N25" s="10"/>
@@ -1537,10 +1528,10 @@
       <c r="I26" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J26" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="K26" s="9"/>
+      <c r="J26" s="15"/>
+      <c r="K26" s="9" t="s">
+        <v>11</v>
+      </c>
       <c r="L26" s="9"/>
       <c r="M26" s="9"/>
       <c r="N26" s="10"/>
@@ -1566,8 +1557,10 @@
       <c r="I27" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J27" s="9"/>
-      <c r="K27" s="9"/>
+      <c r="J27" s="15"/>
+      <c r="K27" s="9" t="s">
+        <v>12</v>
+      </c>
       <c r="L27" s="9"/>
       <c r="M27" s="9"/>
       <c r="N27" s="10"/>
@@ -1591,7 +1584,7 @@
         <v>11</v>
       </c>
       <c r="I28" s="9"/>
-      <c r="J28" s="9"/>
+      <c r="J28" s="15"/>
       <c r="K28" s="9"/>
       <c r="L28" s="9"/>
       <c r="M28" s="9"/>

</xml_diff>